<commit_message>
sprint 4 provisional done
</commit_message>
<xml_diff>
--- a/presentations/links/sprintbacklog4.xlsx
+++ b/presentations/links/sprintbacklog4.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="28810"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="18528"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yathanvidyananthan/Desktop/cscc01/L01_03/presentations/links/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yinli\Programming\CSCC01Repo\L01_03\presentations\links\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="16980"/>
+    <workbookView xWindow="0" yWindow="465" windowWidth="28800" windowHeight="16980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Plan and Sprint Report" sheetId="5" r:id="rId1"/>
     <sheet name="Burndown Chart" sheetId="6" r:id="rId2"/>
     <sheet name="Taskboard Snapshots" sheetId="7" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="150001" concurrentCalc="0"/>
+  <calcPr calcId="171027" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="61">
   <si>
     <t>Task</t>
   </si>
@@ -67,9 +67,6 @@
     <t>As Sohee Kang (professor), I need to create accounts for students and TA's' so that they can access quizzes remotely</t>
   </si>
   <si>
-    <t>As Sohee Kang (professor), I need to create an assignment for each lesson/chapter with the start date and end date</t>
-  </si>
-  <si>
     <t>Provisional:</t>
   </si>
   <si>
@@ -88,27 +85,6 @@
     <t>Create a page for a specific assignment which will list the questions in the assignment</t>
   </si>
   <si>
-    <t>Day 1- Mon Oct 30</t>
-  </si>
-  <si>
-    <t>Day 2- Tues Oct 31</t>
-  </si>
-  <si>
-    <t>Day 3- Wed Nov 1</t>
-  </si>
-  <si>
-    <t>Day 4- Thurs Nov 2</t>
-  </si>
-  <si>
-    <t>Day 5- Fri Nov 3</t>
-  </si>
-  <si>
-    <t>Day 6- Sat Nov 4</t>
-  </si>
-  <si>
-    <t>Day 7- Sun Nov 5</t>
-  </si>
-  <si>
     <t>As Sohee Kang (professor), I need to be able to edit questions and answers after creation</t>
   </si>
   <si>
@@ -121,33 +97,12 @@
     <t>Create a backend call to create student accounts</t>
   </si>
   <si>
-    <t>Create a backend call to create assignments</t>
-  </si>
-  <si>
-    <t>Create a backend call to create questions</t>
-  </si>
-  <si>
-    <t>Create a backend call to edit questions</t>
-  </si>
-  <si>
     <t>Get TA Account creation working with the backend</t>
   </si>
   <si>
     <t>Get Student Account Creation working with the backend</t>
   </si>
   <si>
-    <t>Get assignment creation working with the backend</t>
-  </si>
-  <si>
-    <t>Create a backend call to list assignments</t>
-  </si>
-  <si>
-    <t>Get assignment list to pull data from the backend</t>
-  </si>
-  <si>
-    <t>Create a backend call to list questions</t>
-  </si>
-  <si>
     <t>Create a page to edit questions from</t>
   </si>
   <si>
@@ -166,13 +121,103 @@
     <t>Create a Backend call to accept question responses</t>
   </si>
   <si>
-    <t>Get login pages to poll the login backend</t>
+    <t>Day 1- Mon Nov 06</t>
+  </si>
+  <si>
+    <t>Day 2- Tues Nov 07</t>
+  </si>
+  <si>
+    <t>Day 3- Wed Nov 08</t>
+  </si>
+  <si>
+    <t>Day 4- Thurs Nov 09</t>
+  </si>
+  <si>
+    <t>Day 5- Fri Nov 08</t>
+  </si>
+  <si>
+    <t>Day 6- Sat Nov 10</t>
+  </si>
+  <si>
+    <t>Day 7- Sun Nov 11</t>
+  </si>
+  <si>
+    <t>Same as above</t>
+  </si>
+  <si>
+    <t>We need to be able to create user accounts in the SQL DB for students if the user is logged in with an appropriate session id, and posts the data</t>
+  </si>
+  <si>
+    <t>We need to get the HTML webpage to send the POST request with user data to the Django web app</t>
+  </si>
+  <si>
+    <t>We need an HTML webpage which will list the questions in an assignment and will pull this data from the Django web app</t>
+  </si>
+  <si>
+    <t>We need an HTML webpage which will provide the required forms to create a question, and will send a POST request with data (question, answer, type) from the forms to the Django web app</t>
+  </si>
+  <si>
+    <t>We need an HTML webpage which provides the forms to edit a current Question, and then sends a POST request to the Django web app which will update the SQL DB</t>
+  </si>
+  <si>
+    <t>We need an HTML webpage setup so that it is easily fillable with information from the SQL DB for a single question by the Django web app, and in turn python</t>
+  </si>
+  <si>
+    <t>We need a HTML webpage which is easily fillable with information from the SQL DB for a single short answer question by the Django Web app, and in turn python</t>
+  </si>
+  <si>
+    <t>Create a Django Web App page which when called combines and returns an ajax page filled with information from questions in the SQL DB. The AJAX should come from the templates in tasks 8 and 9.</t>
+  </si>
+  <si>
+    <t>Create an HTML page which will AJAX call the Django web app for a set of questions in an an assignment to be answered, and then provide a button to submit the responses to the Django web APP</t>
+  </si>
+  <si>
+    <t>Create a Django Web App page which will store the question answers for an assignment per user based on POST call from an HTML web page</t>
+  </si>
+  <si>
+    <t>shoaib</t>
+  </si>
+  <si>
+    <t>linhai</t>
+  </si>
+  <si>
+    <t>Calvin</t>
+  </si>
+  <si>
+    <t>Shoaib</t>
+  </si>
+  <si>
+    <t>Linhai</t>
+  </si>
+  <si>
+    <t>Jinming</t>
+  </si>
+  <si>
+    <t>Create a web page to list available assignments</t>
+  </si>
+  <si>
+    <t>We need an HTML webpage setup so that students can see any doable assignments. This will GET info from the Django web app. This page should also lead you into taking the assignment</t>
+  </si>
+  <si>
+    <t>Yathan</t>
+  </si>
+  <si>
+    <t>t5, t6</t>
+  </si>
+  <si>
+    <t>t7, t8</t>
+  </si>
+  <si>
+    <t>t10</t>
+  </si>
+  <si>
+    <t>t11</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -271,7 +316,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -297,9 +342,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -360,7 +402,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -510,7 +552,7 @@
             <c:showPercent val="0"/>
             <c:showBubbleSize val="0"/>
             <c:showLeaderLines val="0"/>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
@@ -536,28 +578,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.0</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.0</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.0</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -569,34 +611,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>18.5</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>16.0</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.0</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.5</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.0</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6.0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.0</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-B8BC-4974-B628-0A342B1B0345}"/>
             </c:ext>
@@ -673,7 +715,7 @@
             <c:showPercent val="0"/>
             <c:showBubbleSize val="0"/>
             <c:showLeaderLines val="0"/>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
@@ -699,28 +741,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.0</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.0</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.0</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -732,34 +774,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>18.5</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18.5</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18.5</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>18.5</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>18.5</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>18.5</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>18.5</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>18.5</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-B8BC-4974-B628-0A342B1B0345}"/>
             </c:ext>
@@ -1005,7 +1047,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="2122075088"/>
-        <c:crossesAt val="1.0"/>
+        <c:crossesAt val="1"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
@@ -1733,7 +1775,7 @@
         <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2038,30 +2080,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Z22"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="53" style="4" customWidth="1"/>
     <col min="3" max="3" width="8" style="4" customWidth="1"/>
-    <col min="4" max="5" width="42.83203125" style="5" customWidth="1"/>
+    <col min="4" max="5" width="42.85546875" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" style="5" customWidth="1"/>
-    <col min="7" max="7" width="8.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="2.83203125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="13.5" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5" style="15" customWidth="1"/>
-    <col min="11" max="11" width="5.83203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="2.85546875" style="3" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" style="14" customWidth="1"/>
+    <col min="11" max="11" width="5.85546875" style="1" customWidth="1"/>
     <col min="12" max="13" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="6" style="1" customWidth="1"/>
     <col min="17" max="17" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.6640625" style="13" customWidth="1"/>
-    <col min="19" max="19" width="7" style="14" customWidth="1"/>
+    <col min="18" max="18" width="3.7109375" style="12" customWidth="1"/>
+    <col min="19" max="19" width="7" style="13" customWidth="1"/>
     <col min="20" max="26" width="6" style="1" customWidth="1"/>
     <col min="27" max="16384" width="12" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:26" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2075,7 +2117,7 @@
         <v>0</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>3</v>
@@ -2086,332 +2128,408 @@
       <c r="I1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="J1" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="S1" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="S1" s="14" t="s">
-        <v>14</v>
-      </c>
       <c r="T1" s="3" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="11">
-        <v>1</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>11</v>
+    <row r="2" spans="1:26" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="9">
+        <v>3</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>15</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="N2" s="1">
-        <v>3</v>
+        <v>17</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="1">
+        <v>2</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="L2" s="1">
+        <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:26" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="9"/>
+      <c r="B3" s="8"/>
       <c r="C3" s="5">
         <v>2</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="P3" s="1">
-        <v>1</v>
+        <v>16</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="1">
+        <v>2</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M3" s="1">
+        <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A4" s="11"/>
-      <c r="B4" s="10"/>
+    <row r="4" spans="1:26" ht="51" x14ac:dyDescent="0.2">
+      <c r="A4" s="9">
+        <v>4</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>18</v>
+      </c>
       <c r="C4" s="5">
         <v>3</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="P4" s="1">
+        <v>24</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G4" s="1">
         <v>1</v>
       </c>
+      <c r="I4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M4" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="5" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="11"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="5">
+    <row r="5" spans="1:26" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="9">
+        <v>5</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="4">
         <v>4</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q5" s="1">
-        <v>1</v>
+        <v>54</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G5" s="1">
+        <v>2</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="O5" s="1">
+        <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A6" s="11"/>
-      <c r="B6" s="10"/>
+    <row r="6" spans="1:26" ht="51" x14ac:dyDescent="0.2">
+      <c r="A6" s="9"/>
+      <c r="B6" s="5"/>
       <c r="C6" s="5">
         <v>5</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q6" s="1">
-        <v>1</v>
+        <v>26</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" s="1">
+        <v>2</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N6" s="1">
+        <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="26" x14ac:dyDescent="0.15">
-      <c r="A7" s="11">
-        <v>2</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>12</v>
-      </c>
+    <row r="7" spans="1:26" ht="51" x14ac:dyDescent="0.2">
       <c r="C7" s="5">
         <v>6</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="N7" s="1">
-        <v>1</v>
-      </c>
-      <c r="P7" s="1">
-        <v>1</v>
+        <v>27</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1">
+        <v>2</v>
+      </c>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="O7" s="1">
+        <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="11"/>
-      <c r="B8" s="12"/>
+    <row r="8" spans="1:26" ht="69" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="5">
         <v>7</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>35</v>
+        <v>28</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="1">
+        <v>2</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="O8" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
+    <row r="9" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
       <c r="C9" s="5">
         <v>8</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="N9" s="1">
+        <v>29</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1">
+        <v>2</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="O9" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="C10" s="5">
+        <v>9</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" s="1">
+        <v>2</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="P10" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="11">
         <v>1</v>
       </c>
-      <c r="P9" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="C10" s="4">
-        <v>9</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="O10" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="38.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="9">
-        <v>3</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>16</v>
+      <c r="B11" s="10" t="s">
+        <v>11</v>
       </c>
       <c r="C11" s="4">
         <v>10</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="P11" s="1">
+      <c r="G11" s="1">
         <v>1</v>
       </c>
+      <c r="I11" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N11" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="12" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="9"/>
-      <c r="B12" s="8"/>
+    <row r="12" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C12" s="5">
         <v>11</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="P12" s="1">
+        <v>20</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G12" s="1">
         <v>1</v>
       </c>
+      <c r="I12" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="N12" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="13" spans="1:26" ht="26" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:26" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A13" s="11"/>
+      <c r="B13" s="10"/>
       <c r="C13" s="5">
         <v>12</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F13" s="1"/>
-      <c r="P13" s="1">
+        <v>22</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" s="1">
+        <v>2</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q13" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A14" s="11"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="5">
+        <v>13</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="1">
+        <v>1</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="51" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="17" spans="7:26" ht="26.1" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="18" spans="7:26" ht="15" x14ac:dyDescent="0.25">
+      <c r="G18" s="2">
+        <f>SUM(G2:G14)</f>
+        <v>22</v>
+      </c>
+      <c r="K18" s="6">
+        <f>SUM(K1:K14)</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="6">
+        <f>SUM(L2:L14)</f>
+        <v>2</v>
+      </c>
+      <c r="M18" s="6">
+        <f t="shared" ref="M18:Q18" si="0">SUM(M2:M14)</f>
         <v>3</v>
       </c>
+      <c r="N18" s="6">
+        <f>SUM(N2:N14)</f>
+        <v>4</v>
+      </c>
+      <c r="O18" s="6">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="P18" s="6">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="Q18" s="6">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="C14" s="4">
-        <v>13</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" s="1"/>
-      <c r="P14" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" ht="51" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="9">
-        <v>4</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="5">
-        <v>14</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A16" s="9"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5">
-        <v>15</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="P16" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="9">
-        <v>5</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" s="5">
-        <v>16</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="M17" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A18" s="9"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5">
-        <v>17</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="M18" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A19" s="9"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5">
-        <v>18</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>43</v>
-      </c>
+    <row r="19" spans="7:26" x14ac:dyDescent="0.2">
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
-      <c r="P19" s="1">
-        <v>2</v>
-      </c>
       <c r="Q19" s="2"/>
       <c r="Z19" s="2"/>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A20" s="9"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5">
-        <v>19</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="P20" s="1">
-        <v>2</v>
-      </c>
+    <row r="20" spans="7:26" x14ac:dyDescent="0.2">
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
@@ -2419,56 +2537,7 @@
       <c r="X20" s="2"/>
       <c r="Y20" s="2"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="C21" s="5">
-        <v>20</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="M21" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="24" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="G24" s="2">
-        <f>SUM(G2:G23)</f>
-        <v>0</v>
-      </c>
-      <c r="K24" s="6">
-        <f>SUM(K2:K22)</f>
-        <v>0</v>
-      </c>
-      <c r="L24" s="6">
-        <f t="shared" ref="L24:Q24" si="0">SUM(L2:L22)</f>
-        <v>0</v>
-      </c>
-      <c r="M24" s="6">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="N24" s="6">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="O24" s="6">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="P24" s="6">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="Q24" s="6">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.15">
-      <c r="A33" s="9"/>
-      <c r="B33" s="5"/>
-    </row>
+    <row r="22" spans="7:26" ht="26.1" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="R1:R1048576"/>
@@ -2481,30 +2550,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="3" width="4.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
+    <col min="2" max="3" width="4.85546875" customWidth="1"/>
     <col min="4" max="4" width="5" customWidth="1"/>
-    <col min="5" max="9" width="4.83203125" customWidth="1"/>
+    <col min="5" max="9" width="4.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
@@ -2533,74 +2602,74 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
       <c r="B3">
-        <v>18.5</v>
+        <v>22</v>
       </c>
       <c r="C3">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D3">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="E3">
-        <v>7.5</v>
+        <v>17</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="G3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
       <c r="B4">
-        <v>18.5</v>
+        <v>22</v>
       </c>
       <c r="C4">
-        <v>18.5</v>
+        <v>22</v>
       </c>
       <c r="D4">
-        <v>18.5</v>
+        <v>22</v>
       </c>
       <c r="E4">
-        <v>18.5</v>
+        <v>22</v>
       </c>
       <c r="F4">
-        <v>18.5</v>
+        <v>22</v>
       </c>
       <c r="G4">
-        <v>18.5</v>
+        <v>22</v>
       </c>
       <c r="H4">
-        <v>18.5</v>
+        <v>22</v>
       </c>
       <c r="I4">
-        <v>18.5</v>
+        <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2614,9 +2683,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2624,14 +2693,54 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?><ct:contentTypeSchema ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F770ABC8F9B27C4C8461F4575C23FAEA" ma:contentTypeVersion="1" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6f0f4afd6cc55b40f57cb0d59e49aa45" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes">
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?><p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"><documentManagement><_dlc_DocId xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07">WORK-769-153</_dlc_DocId><_dlc_DocIdUrl xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07"><Url>http://intranet/workingtogether/projects/110405/_layouts/DocIdRedir.aspx?ID=WORK-769-153</Url><Description>WORK-769-153</Description></_dlc_DocIdUrl><IconOverlay xmlns="http://schemas.microsoft.com/sharepoint/v4" xsi:nil="true"/><Last_x0020_Archive xmlns="$ListId:Shared Documents;" xsi:nil="true"/><Reason xmlns="$ListId:Shared Documents;" xsi:nil="true"></Reason></documentManagement></p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?><ct:contentTypeSchema ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F770ABC8F9B27C4C8461F4575C23FAEA" ma:contentTypeVersion="1" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6f0f4afd6cc55b40f57cb0d59e49aa45" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes">
 <xsd:schema targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f7c28edf12e174e47f2c7bd2736e8bd" ns2:_="" ns3:_="" ns4:_="" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d93dc7d-5998-434b-bf34-aa89b432ec07" xmlns:ns3="$ListId:Shared Documents;" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v4">
 <xsd:import namespace="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
 <xsd:import namespace="$ListId:Shared Documents;"/>
@@ -2805,64 +2914,36 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?><p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"><documentManagement><_dlc_DocId xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07">WORK-769-153</_dlc_DocId><_dlc_DocIdUrl xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07"><Url>http://intranet/workingtogether/projects/110405/_layouts/DocIdRedir.aspx?ID=WORK-769-153</Url><Description>WORK-769-153</Description></_dlc_DocIdUrl><IconOverlay xmlns="http://schemas.microsoft.com/sharepoint/v4" xsi:nil="true"/><Last_x0020_Archive xmlns="$ListId:Shared Documents;" xsi:nil="true"/><Reason xmlns="$ListId:Shared Documents;" xsi:nil="true"></Reason></documentManagement></p:properties>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B9EEEF-7393-4E57-9716-D967A23AC816}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F807D2B-FCE5-4B63-BC9A-551BEF173D66}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47BCCC64-3980-40D2-8C4F-F5BACE67ECB4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v4"/>
+    <ds:schemaRef ds:uri="$ListId:Shared Documents;"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0008E140-BD0E-4C41-947D-F18B1A1E4B6B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2882,22 +2963,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47BCCC64-3980-40D2-8C4F-F5BACE67ECB4}">
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B9EEEF-7393-4E57-9716-D967A23AC816}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v4"/>
-    <ds:schemaRef ds:uri="$ListId:Shared Documents;"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F807D2B-FCE5-4B63-BC9A-551BEF173D66}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>